<commit_message>
exp strat eval 08-30-3-v2
</commit_message>
<xml_diff>
--- a/results/reliability_eval/unified_scores_table_08-30-3.xlsx
+++ b/results/reliability_eval/unified_scores_table_08-30-3.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P6"/>
+  <dimension ref="A1:P11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -698,12 +698,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>toy-qa-dataset</t>
+          <t>P101</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>neg2</t>
+          <t>neg1</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -713,41 +713,41 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>beam</t>
+          <t>sample</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="G5" t="n">
         <v>0.1</v>
       </c>
       <c r="H5" t="n">
-        <v>0.5714285714285714</v>
+        <v>0.26</v>
       </c>
       <c r="I5" t="n">
-        <v>0.8425925925925926</v>
+        <v>0.6325363825363826</v>
       </c>
       <c r="J5" t="n">
-        <v>0.8283399470899472</v>
+        <v>0.3437088412498248</v>
       </c>
       <c r="K5" t="n">
-        <v>0.8425925925925926</v>
+        <v>0.6325363825363826</v>
       </c>
       <c r="L5" t="n">
-        <v>0.8283399470899472</v>
+        <v>0.3437088412498248</v>
       </c>
       <c r="M5" t="n">
-        <v>0.212962962962963</v>
+        <v>0.3653846153846154</v>
       </c>
       <c r="N5" t="n">
-        <v>0.4547508004551349</v>
+        <v>0.2558704453441296</v>
       </c>
       <c r="O5" t="n">
-        <v>1</v>
+        <v>0.9937629937629937</v>
       </c>
       <c r="P5" t="n">
-        <v>1</v>
+        <v>0.9692307692307692</v>
       </c>
     </row>
     <row r="6">
@@ -758,12 +758,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>toy-qa-dataset</t>
+          <t>P101</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>neg2</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -773,41 +773,341 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>beam</t>
+          <t>sample</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="G6" t="n">
         <v>0.1</v>
       </c>
       <c r="H6" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.3276190476190476</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.2508664315689825</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.3276190476190476</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.2508664315689825</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0.6257142857142857</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0.3628220985363843</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0.980952380952381</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Llama-3-8B</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>toy-qa-dataset</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>neg2</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>fact_statement</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>beam</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>10</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.8425925925925926</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.8283399470899472</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0.8425925925925926</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.8283399470899472</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0.212962962962963</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0.4547508004551349</v>
+      </c>
+      <c r="O7" t="n">
+        <v>1</v>
+      </c>
+      <c r="P7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Llama-3-8B</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>P101</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>neg3</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>fact_statement</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>sample</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>20</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.5762499999999999</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.2392696858425133</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0.5762499999999999</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.2392696858425133</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0.1804651162790697</v>
+      </c>
+      <c r="O8" t="n">
+        <v>1</v>
+      </c>
+      <c r="P8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Llama-3-8B</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>toy-qa-dataset</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>fact_statement</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>beam</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>10</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H9" t="n">
         <v>0.7619047619047619</v>
       </c>
-      <c r="I6" t="n">
+      <c r="I9" t="n">
         <v>0.975</v>
       </c>
-      <c r="J6" t="n">
+      <c r="J9" t="n">
         <v>0.9930555555555556</v>
       </c>
-      <c r="K6" t="n">
+      <c r="K9" t="n">
         <v>0.975</v>
       </c>
-      <c r="L6" t="n">
+      <c r="L9" t="n">
         <v>0.9930555555555556</v>
       </c>
-      <c r="M6" t="n">
+      <c r="M9" t="n">
         <v>0.225</v>
       </c>
-      <c r="N6" t="n">
+      <c r="N9" t="n">
         <v>0.6500599549336971</v>
       </c>
-      <c r="O6" t="n">
-        <v>1</v>
-      </c>
-      <c r="P6" t="n">
-        <v>1</v>
+      <c r="O9" t="n">
+        <v>1</v>
+      </c>
+      <c r="P9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Llama-3-8B</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>P101</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>fact_statement</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>sample</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>20</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.525</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.225</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0.525</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.225</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0.2470588235294118</v>
+      </c>
+      <c r="O10" t="n">
+        <v>1</v>
+      </c>
+      <c r="P10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Llama-3-8B</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>P101</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>pos</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>fact_statement</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>sample</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>20</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.02445652173913042</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.05580013736263736</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0.02445652173913042</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0.05580013736263736</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0.9836956521739131</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0.8178571428571428</v>
+      </c>
+      <c r="O11" t="n">
+        <v>0.9891304347826088</v>
+      </c>
+      <c r="P11" t="n">
+        <v>0.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>